<commit_message>
Update reports and add Kenya X/TikTok/Instagram engagement coverage + scrapers
</commit_message>
<xml_diff>
--- a/Research Assets/Engagement Metrics/Nigeria/Engagement ContentAnalysis Merged.xlsx
+++ b/Research Assets/Engagement Metrics/Nigeria/Engagement ContentAnalysis Merged.xlsx
@@ -578,10 +578,8 @@
           <t>https://x.com/_deyemi/status/1862512830987346178</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1862512830987346178</t>
-        </is>
+      <c r="F2" t="n">
+        <v>1.862512830987346e+18</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -684,10 +682,8 @@
           <t>https://x.com/_deyemi/status/1848028499606380555</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1848028499606380555</t>
-        </is>
+      <c r="F3" t="n">
+        <v>1.848028499606381e+18</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -790,10 +786,8 @@
           <t>https://x.com/_deyemi/status/1846206865396347176</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1846206865396347176</t>
-        </is>
+      <c r="F4" t="n">
+        <v>1.846206865396347e+18</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,10 +890,8 @@
           <t>https://x.com/_deyemi/status/1694030169491538367</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1694030169491538367</t>
-        </is>
+      <c r="F5" t="n">
+        <v>1.694030169491538e+18</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1002,10 +994,8 @@
           <t>https://x.com/_deyemi/status/1674519625365876736</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1674519625365876736</t>
-        </is>
+      <c r="F6" t="n">
+        <v>1.674519625365877e+18</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1108,10 +1098,8 @@
           <t>https://x.com/_deyemi/status/1660336229508870151</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1660336229508870151</t>
-        </is>
+      <c r="F7" t="n">
+        <v>1.66033622950887e+18</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1214,10 +1202,8 @@
           <t>https://x.com/_deyemi/status/1640650926959599618</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>1640650926959599618</t>
-        </is>
+      <c r="F8" t="n">
+        <v>1.6406509269596e+18</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1320,10 +1306,8 @@
           <t>https://x.com/_deyemi/status/1640369752345288706</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1640369752345288706</t>
-        </is>
+      <c r="F9" t="n">
+        <v>1.640369752345289e+18</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1426,10 +1410,8 @@
           <t>https://x.com/_deyemi/status/1612001517711523841</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1612001517711523841</t>
-        </is>
+      <c r="F10" t="n">
+        <v>1.612001517711524e+18</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1532,10 +1514,8 @@
           <t>https://x.com/_deyemi/status/1226450923859464193</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1226450923859464193</t>
-        </is>
+      <c r="F11" t="n">
+        <v>1.226450923859464e+18</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1603,7 +1583,6 @@
       <c r="V11" t="n">
         <v>0</v>
       </c>
-      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
         <is>
           <t>Sun Feb 09 10:21:01 +0000 2020</t>
@@ -1636,10 +1615,8 @@
           <t>https://x.com/_deyemi/status/1226493015319105537</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1226493015319105537</t>
-        </is>
+      <c r="F12" t="n">
+        <v>1.226493015319106e+18</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1707,7 +1684,6 @@
       <c r="V12" t="n">
         <v>0</v>
       </c>
-      <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
           <t>Sun Feb 09 13:08:16 +0000 2020</t>
@@ -1740,10 +1716,8 @@
           <t>https://x.com/_deyemi/status/1309190324355563521</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1309190324355563521</t>
-        </is>
+      <c r="F13" t="n">
+        <v>1.309190324355564e+18</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1811,7 +1785,6 @@
       <c r="V13" t="n">
         <v>0</v>
       </c>
-      <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr">
         <is>
           <t>Thu Sep 24 17:57:51 +0000 2020</t>
@@ -1844,10 +1817,8 @@
           <t>https://x.com/_deyemi/status/1309679015171698690</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1309679015171698690</t>
-        </is>
+      <c r="F14" t="n">
+        <v>1.309679015171699e+18</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1901,7 +1872,7 @@
         </is>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
@@ -1915,7 +1886,6 @@
       <c r="V14" t="n">
         <v>0</v>
       </c>
-      <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr">
         <is>
           <t>Fri Sep 25 23:16:29 +0000 2020</t>
@@ -1948,10 +1918,8 @@
           <t>https://x.com/_deyemi/status/1333661251948441600</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1333661251948441600</t>
-        </is>
+      <c r="F15" t="n">
+        <v>1.333661251948442e+18</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -2019,7 +1987,6 @@
       <c r="V15" t="n">
         <v>0</v>
       </c>
-      <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr">
         <is>
           <t>Mon Nov 30 22:57:39 +0000 2020</t>
@@ -2052,10 +2019,8 @@
           <t>https://x.com/_deyemi/status/1396817067316289537</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>1396817067316289537</t>
-        </is>
+      <c r="F16" t="n">
+        <v>1.39681706731629e+18</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -2109,13 +2074,13 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -2123,7 +2088,6 @@
       <c r="V16" t="n">
         <v>0</v>
       </c>
-      <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr">
         <is>
           <t>Mon May 24 13:11:25 +0000 2021</t>
@@ -2156,10 +2120,8 @@
           <t>https://x.com/_deyemi/status/1396816102240489479</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>1396816102240489479</t>
-        </is>
+      <c r="F17" t="n">
+        <v>1.396816102240489e+18</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2227,7 +2189,6 @@
       <c r="V17" t="n">
         <v>0</v>
       </c>
-      <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr">
         <is>
           <t>Mon May 24 13:11:25 +0000 2021</t>
@@ -2260,10 +2221,8 @@
           <t>https://x.com/_deyemi/status/1484112712443518978</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>1484112712443518978</t>
-        </is>
+      <c r="F18" t="n">
+        <v>1.484112712443519e+18</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2331,7 +2290,6 @@
       <c r="V18" t="n">
         <v>0</v>
       </c>
-      <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr">
         <is>
           <t>Thu Jan 20 10:36:58 +0000 2022</t>
@@ -2364,10 +2322,8 @@
           <t>https://x.com/_deyemi/status/1558235509062770688</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>1558235509062770688</t>
-        </is>
+      <c r="F19" t="n">
+        <v>1.558235509062771e+18</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -2379,15 +2335,6 @@
           <t>Deyemi Okanlawon questions the assumption that men are solely providers in marriage, using a rhetorical question and a smiley face.</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="n">
         <v>0</v>
       </c>
@@ -2403,7 +2350,6 @@
       <c r="V19" t="n">
         <v>0</v>
       </c>
-      <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr">
         <is>
           <t>Thu Aug 11 09:35:26 +0000 2022</t>
@@ -2436,10 +2382,8 @@
           <t>https://x.com/_deyemi/status/1557661960992428032</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>1557661960992428032</t>
-        </is>
+      <c r="F20" t="n">
+        <v>1.557661960992428e+18</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2451,23 +2395,14 @@
           <t>Deyemi Okanlawon warns men about stress-related health risks, criticizing societal pressure on men as sole providers; 'provider' implies traditional male role.</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>6246</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>2143</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -2475,7 +2410,6 @@
       <c r="V20" t="n">
         <v>0</v>
       </c>
-      <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr">
         <is>
           <t>Thu Aug 11 09:35:26 +0000 2022</t>
@@ -2508,10 +2442,8 @@
           <t>https://x.com/_deyemi/status/1852709730671636910</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1852709730671636910</t>
-        </is>
+      <c r="F21" t="n">
+        <v>1.852709730671637e+18</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2524,15 +2456,6 @@
           <t>Deyemi Okanlawon discusses the difficulty men face in showing vulnerability due to societal pressures, choosing to confront internal struggles openly.</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="n">
         <v>93</v>
       </c>
@@ -2583,10 +2506,8 @@
           <t>https://x.com/_deyemi/status/1901981220218577289</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>1901981220218577289</t>
-        </is>
+      <c r="F22" t="n">
+        <v>1.901981220218577e+18</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2598,15 +2519,6 @@
           <t>Deyemi Okanlawon expresses emotional difficulty watching a Netflix show about adolescence, fearing its relevance to his experience as a father of three sons.</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="n">
         <v>21</v>
       </c>
@@ -2657,10 +2569,8 @@
           <t>https://x.com/_deyemi/status/1991944018058727780</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>1991944018058727780</t>
-        </is>
+      <c r="F23" t="n">
+        <v>1.991944018058728e+18</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2672,15 +2582,6 @@
           <t>Deyemi Okanlawon emphasizes checking in on friends' well-being beyond surface-level responses, using 'abeg' (Pidgin for 'please') to stress importance.</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
         <v>182</v>
       </c>
@@ -2731,10 +2632,8 @@
           <t>https://x.com/_deyemi/status/1594672742464622592</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>1594672742464622592</t>
-        </is>
+      <c r="F24" t="n">
+        <v>1.594672742464623e+18</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2746,15 +2645,6 @@
           <t>Deyemi Okanlawon expresses his aspiration to fulfill various personal and social roles, acknowledging his imperfections and seeking divine assistance.</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="n">
         <v>228</v>
       </c>
@@ -2770,7 +2660,6 @@
       <c r="V24" t="n">
         <v>0</v>
       </c>
-      <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr">
         <is>
           <t>Mon Nov 21 12:43:04 +0000 2022</t>
@@ -2803,10 +2692,8 @@
           <t>https://x.com/_deyemi/status/1380908200388661256</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>1380908200388661256</t>
-        </is>
+      <c r="F25" t="n">
+        <v>1.380908200388661e+18</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2818,15 +2705,6 @@
           <t>Deyemi Okanlawon criticizes backlash against Chimamanda, highlighting misunderstandings and condemning cancel culture and online bullying.</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="n">
         <v>30</v>
       </c>
@@ -2842,7 +2720,6 @@
       <c r="V25" t="n">
         <v>0</v>
       </c>
-      <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr">
         <is>
           <t>Sat Apr 10 15:39:05 +0000 2021</t>
@@ -2875,10 +2752,8 @@
           <t>https://x.com/_deyemi/status/1223908274380079107</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>1223908274380079107</t>
-        </is>
+      <c r="F26" t="n">
+        <v>1.223908274380079e+18</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2890,15 +2765,6 @@
           <t>The tweet critiques the misuse of the phrase 'not all men' while advocating for equal rights and opportunities for all individuals.</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="n">
         <v>1</v>
       </c>
@@ -2914,7 +2780,6 @@
       <c r="V26" t="n">
         <v>0</v>
       </c>
-      <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr">
         <is>
           <t>Sun Feb 02 09:57:26 +0000 2020</t>
@@ -2947,10 +2812,8 @@
           <t>https://x.com/_deyemi/status/1606029138787151873</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>1606029138787151873</t>
-        </is>
+      <c r="F27" t="n">
+        <v>1.606029138787152e+18</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2962,15 +2825,6 @@
           <t>A prayer for personal growth and marital harmony, inspired by a desire to emulate a positive example seen in a video.</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="n">
         <v>44</v>
       </c>
@@ -3021,10 +2875,8 @@
           <t>https://x.com/itsSh0la/status/1664024839475335168</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>1664024839475335168</t>
-        </is>
+      <c r="F28" t="n">
+        <v>1.664024839475335e+18</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3127,10 +2979,8 @@
           <t>https://x.com/itsSh0la/status/1664019236597932032</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>1664019236597932032</t>
-        </is>
+      <c r="F29" t="n">
+        <v>1.664019236597932e+18</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3184,7 +3034,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>7596</v>
       </c>
       <c r="S29" t="n">
         <v>0</v>
@@ -3233,10 +3083,8 @@
           <t>https://x.com/itsSh0la/status/1663625331905904641</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>1663625331905904641</t>
-        </is>
+      <c r="F30" t="n">
+        <v>1.663625331905905e+18</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -3339,10 +3187,8 @@
           <t>https://x.com/itsSh0la/status/1662863528896745472</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>1662863528896745472</t>
-        </is>
+      <c r="F31" t="n">
+        <v>1.662863528896745e+18</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -3396,7 +3242,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>9842</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
@@ -3445,10 +3291,8 @@
           <t>https://x.com/itsSh0la/status/1662499938104754176</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>1662499938104754176</t>
-        </is>
+      <c r="F32" t="n">
+        <v>1.662499938104754e+18</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -3502,7 +3346,7 @@
         </is>
       </c>
       <c r="R32" t="n">
-        <v>0</v>
+        <v>2369</v>
       </c>
       <c r="S32" t="n">
         <v>0</v>
@@ -3551,10 +3395,8 @@
           <t>https://x.com/itsSh0la/status/1662402106442104832</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>1662402106442104832</t>
-        </is>
+      <c r="F33" t="n">
+        <v>1.662402106442105e+18</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3657,10 +3499,8 @@
           <t>https://x.com/itsSh0la/status/1662139482320125979</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>1662139482320125979</t>
-        </is>
+      <c r="F34" t="n">
+        <v>1.662139482320126e+18</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -3714,7 +3554,7 @@
         </is>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>4312</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
@@ -3763,10 +3603,8 @@
           <t>https://x.com/itsSh0la/status/1661717784420655104</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>1661717784420655104</t>
-        </is>
+      <c r="F35" t="n">
+        <v>1.661717784420655e+18</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -3869,10 +3707,8 @@
           <t>https://x.com/itsSh0la/status/1661677741761089540</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>1661677741761089540</t>
-        </is>
+      <c r="F36" t="n">
+        <v>1.66167774176109e+18</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3975,10 +3811,8 @@
           <t>https://x.com/itsSh0la/status/1652790345598418944</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>1652790345598418944</t>
-        </is>
+      <c r="F37" t="n">
+        <v>1.652790345598419e+18</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -4032,13 +3866,13 @@
         </is>
       </c>
       <c r="R37" t="n">
-        <v>0</v>
+        <v>3780</v>
       </c>
       <c r="S37" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="T37" t="n">
-        <v>0</v>
+        <v>574</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -4081,10 +3915,8 @@
           <t>https://x.com/itsSh0la/status/1652785564301635587</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>1652785564301635587</t>
-        </is>
+      <c r="F38" t="n">
+        <v>1.652785564301636e+18</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -4187,10 +4019,8 @@
           <t>https://x.com/itsSh0la/status/1652627388813959168</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>1652627388813959168</t>
-        </is>
+      <c r="F39" t="n">
+        <v>1.652627388813959e+18</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -4293,10 +4123,8 @@
           <t>https://x.com/itsSh0la/status/1652263110000926720</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>1652263110000926720</t>
-        </is>
+      <c r="F40" t="n">
+        <v>1.652263110000927e+18</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -4399,10 +4227,8 @@
           <t>https://x.com/itsSh0la/status/1652003604738220032</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>1652003604738220032</t>
-        </is>
+      <c r="F41" t="n">
+        <v>1.65200360473822e+18</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -4505,10 +4331,8 @@
           <t>https://x.com/itsSh0la/status/1652003600707534862</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>1652003600707534862</t>
-        </is>
+      <c r="F42" t="n">
+        <v>1.652003600707535e+18</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -4611,10 +4435,8 @@
           <t>https://x.com/itsSh0la/status/1652003596555173910</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>1652003596555173910</t>
-        </is>
+      <c r="F43" t="n">
+        <v>1.652003596555174e+18</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -4717,10 +4539,8 @@
           <t>https://x.com/itsSh0la/status/1652003592700608534</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>1652003592700608534</t>
-        </is>
+      <c r="F44" t="n">
+        <v>1.652003592700609e+18</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -4823,10 +4643,8 @@
           <t>https://x.com/itsSh0la/status/1652003588904828930</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>1652003588904828930</t>
-        </is>
+      <c r="F45" t="n">
+        <v>1.652003588904829e+18</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -4929,10 +4747,8 @@
           <t>https://x.com/itsSh0la/status/1652003585423491082</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>1652003585423491082</t>
-        </is>
+      <c r="F46" t="n">
+        <v>1.652003585423491e+18</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -5035,10 +4851,8 @@
           <t>https://x.com/itsSh0la/status/1651950305637027840</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>1651950305637027840</t>
-        </is>
+      <c r="F47" t="n">
+        <v>1.651950305637028e+18</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -5141,10 +4955,8 @@
           <t>https://x.com/itsSh0la/status/1651922915389059073</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>1651922915389059073</t>
-        </is>
+      <c r="F48" t="n">
+        <v>1.651922915389059e+18</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -5247,10 +5059,8 @@
           <t>https://x.com/itsSh0la/status/1651920790151995392</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>1651920790151995392</t>
-        </is>
+      <c r="F49" t="n">
+        <v>1.651920790151995e+18</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -5353,10 +5163,8 @@
           <t>https://x.com/itsSh0la/status/1651911094334550016</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>1651911094334550016</t>
-        </is>
+      <c r="F50" t="n">
+        <v>1.65191109433455e+18</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -5459,10 +5267,8 @@
           <t>https://x.com/itsSh0la/status/1651564511965454342</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>1651564511965454342</t>
-        </is>
+      <c r="F51" t="n">
+        <v>1.651564511965454e+18</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -5565,10 +5371,8 @@
           <t>https://x.com/itsSh0la/status/1651213879349747712</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>1651213879349747712</t>
-        </is>
+      <c r="F52" t="n">
+        <v>1.651213879349748e+18</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -5622,13 +5426,13 @@
         </is>
       </c>
       <c r="R52" t="n">
-        <v>0</v>
+        <v>7524</v>
       </c>
       <c r="S52" t="n">
-        <v>0</v>
+        <v>974</v>
       </c>
       <c r="T52" t="n">
-        <v>0</v>
+        <v>848</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -5671,10 +5475,8 @@
           <t>https://x.com/itsSh0la/status/1651167539420954624</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>1651167539420954624</t>
-        </is>
+      <c r="F53" t="n">
+        <v>1.651167539420955e+18</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -5777,10 +5579,8 @@
           <t>https://x.com/itsSh0la/status/1651167535662788610</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>1651167535662788610</t>
-        </is>
+      <c r="F54" t="n">
+        <v>1.651167535662789e+18</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -5883,10 +5683,8 @@
           <t>https://x.com/itsSh0la/status/1651167532152246280</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>1651167532152246280</t>
-        </is>
+      <c r="F55" t="n">
+        <v>1.651167532152246e+18</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -5989,10 +5787,8 @@
           <t>https://x.com/itsSh0la/status/1651167528620630016</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>1651167528620630016</t>
-        </is>
+      <c r="F56" t="n">
+        <v>1.65116752862063e+18</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -6095,10 +5891,8 @@
           <t>https://x.com/itsSh0la/status/1651167524862451713</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>1651167524862451713</t>
-        </is>
+      <c r="F57" t="n">
+        <v>1.651167524862452e+18</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -6201,10 +5995,8 @@
           <t>https://x.com/itsSh0la/status/1651167521314156544</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>1651167521314156544</t>
-        </is>
+      <c r="F58" t="n">
+        <v>1.651167521314157e+18</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -6307,10 +6099,8 @@
           <t>https://x.com/itsSh0la/status/1651167515811233795</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>1651167515811233795</t>
-        </is>
+      <c r="F59" t="n">
+        <v>1.651167515811234e+18</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -6413,10 +6203,8 @@
           <t>https://x.com/itsSh0la/status/1651167509154807810</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>1651167509154807810</t>
-        </is>
+      <c r="F60" t="n">
+        <v>1.651167509154808e+18</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -6519,10 +6307,8 @@
           <t>https://x.com/itsSh0la/status/1650962741857775634</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>1650962741857775634</t>
-        </is>
+      <c r="F61" t="n">
+        <v>1.650962741857776e+18</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -6625,10 +6411,8 @@
           <t>https://x.com/itsSh0la/status/1641505314150162433</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>1641505314150162433</t>
-        </is>
+      <c r="F62" t="n">
+        <v>1.641505314150162e+18</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -6731,10 +6515,8 @@
           <t>https://x.com/itsSh0la/status/1641439108915425280</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>1641439108915425280</t>
-        </is>
+      <c r="F63" t="n">
+        <v>1.641439108915425e+18</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -6837,10 +6619,8 @@
           <t>https://x.com/itsSh0la/status/1641094628173643778</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>1641094628173643778</t>
-        </is>
+      <c r="F64" t="n">
+        <v>1.641094628173644e+18</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -6943,10 +6723,8 @@
           <t>https://x.com/itsSh0la/status/1641094150786367489</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>1641094150786367489</t>
-        </is>
+      <c r="F65" t="n">
+        <v>1.641094150786367e+18</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -7049,10 +6827,8 @@
           <t>https://x.com/itsSh0la/status/1641089707684536320</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>1641089707684536320</t>
-        </is>
+      <c r="F66" t="n">
+        <v>1.641089707684536e+18</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -7155,10 +6931,8 @@
           <t>https://x.com/itsSh0la/status/1640845160861908993</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>1640845160861908993</t>
-        </is>
+      <c r="F67" t="n">
+        <v>1.640845160861909e+18</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -7261,10 +7035,8 @@
           <t>https://x.com/itsSh0la/status/1640435905209966597</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>1640435905209966597</t>
-        </is>
+      <c r="F68" t="n">
+        <v>1.640435905209967e+18</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -7367,10 +7139,8 @@
           <t>https://x.com/itsSh0la/status/1628468754609831944</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>1628468754609831944</t>
-        </is>
+      <c r="F69" t="n">
+        <v>1.628468754609832e+18</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -7473,10 +7243,8 @@
           <t>https://x.com/itsSh0la/status/1628463098209177603</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>1628463098209177603</t>
-        </is>
+      <c r="F70" t="n">
+        <v>1.628463098209178e+18</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -7579,10 +7347,8 @@
           <t>https://x.com/itsSh0la/status/1628416830455877634</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>1628416830455877634</t>
-        </is>
+      <c r="F71" t="n">
+        <v>1.628416830455878e+18</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -7685,10 +7451,8 @@
           <t>https://x.com/itsSh0la/status/1628416198659526656</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>1628416198659526656</t>
-        </is>
+      <c r="F72" t="n">
+        <v>1.628416198659527e+18</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -7791,10 +7555,8 @@
           <t>https://x.com/itsSh0la/status/1628159921660256256</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>1628159921660256256</t>
-        </is>
+      <c r="F73" t="n">
+        <v>1.628159921660256e+18</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -7897,10 +7659,8 @@
           <t>https://x.com/itsSh0la/status/1662051837590077440</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>1662051837590077440</t>
-        </is>
+      <c r="F74" t="n">
+        <v>1.662051837590077e+18</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -8003,10 +7763,8 @@
           <t>https://x.com/itsSh0la/status/1650853184552980485</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>1650853184552980485</t>
-        </is>
+      <c r="F75" t="n">
+        <v>1.65085318455298e+18</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -8109,10 +7867,8 @@
           <t>https://x.com/itsSh0la/status/1641175498410672130</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>1641175498410672130</t>
-        </is>
+      <c r="F76" t="n">
+        <v>1.641175498410672e+18</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -8215,10 +7971,8 @@
           <t>https://x.com/itsSh0la/status/1628509804153929742</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>1628509804153929742</t>
-        </is>
+      <c r="F77" t="n">
+        <v>1.62850980415393e+18</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -8321,10 +8075,8 @@
           <t>https://x.com/itsSh0la/status/1628469143472144385</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>1628469143472144385</t>
-        </is>
+      <c r="F78" t="n">
+        <v>1.628469143472144e+18</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -8427,10 +8179,8 @@
           <t>https://x.com/itsSh0la/status/1628156373774090243</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>1628156373774090243</t>
-        </is>
+      <c r="F79" t="n">
+        <v>1.62815637377409e+18</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -8533,10 +8283,8 @@
           <t>https://x.com/itsSh0la/status/1627968217946759170</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>1627968217946759170</t>
-        </is>
+      <c r="F80" t="n">
+        <v>1.627968217946759e+18</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -8639,10 +8387,8 @@
           <t>https://x.com/itsSh0la/status/1627951140041097218</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>1627951140041097218</t>
-        </is>
+      <c r="F81" t="n">
+        <v>1.627951140041097e+18</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -8696,10 +8442,10 @@
         </is>
       </c>
       <c r="R81" t="n">
-        <v>0</v>
+        <v>5511</v>
       </c>
       <c r="S81" t="n">
-        <v>0</v>
+        <v>1017</v>
       </c>
       <c r="T81" t="n">
         <v>0</v>
@@ -8745,10 +8491,8 @@
           <t>https://x.com/itsSh0la/status/1627951136610086912</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>1627951136610086912</t>
-        </is>
+      <c r="F82" t="n">
+        <v>1.627951136610087e+18</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -8851,10 +8595,8 @@
           <t>https://x.com/itsSh0la/status/1627951132671606784</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>1627951132671606784</t>
-        </is>
+      <c r="F83" t="n">
+        <v>1.627951132671607e+18</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -8957,10 +8699,8 @@
           <t>https://x.com/itsSh0la/status/1627942731166150657</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>1627942731166150657</t>
-        </is>
+      <c r="F84" t="n">
+        <v>1.627942731166151e+18</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -9063,10 +8803,8 @@
           <t>https://x.com/itsSh0la/status/1627942727752069120</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>1627942727752069120</t>
-        </is>
+      <c r="F85" t="n">
+        <v>1.627942727752069e+18</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -9169,10 +8907,8 @@
           <t>https://x.com/itsSh0la/status/1627942720940433413</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>1627942720940433413</t>
-        </is>
+      <c r="F86" t="n">
+        <v>1.627942720940433e+18</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -9275,10 +9011,8 @@
           <t>https://x.com/itsSh0la/status/1627942717320843271</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>1627942717320843271</t>
-        </is>
+      <c r="F87" t="n">
+        <v>1.627942717320843e+18</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -9290,15 +9024,6 @@
           <t>A man was blocked by his girlfriend after gifting her, as she preferred another who bought her friend an iPhone 14.</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
       <c r="R87" t="n">
         <v>5511</v>
       </c>
@@ -9349,10 +9074,8 @@
           <t>https://x.com/itsSh0la/status/1627281039818207234</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>1627281039818207234</t>
-        </is>
+      <c r="F88" t="n">
+        <v>1.627281039818207e+18</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -9364,15 +9087,6 @@
           <t>The text critiques the notion of 'independent woman' by comparing it to a man claiming independence, suggesting self-sufficiency is a basic adult responsibility.</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
       <c r="R88" t="n">
         <v>7254</v>
       </c>
@@ -9423,10 +9137,8 @@
           <t>https://x.com/itsSh0la/status/1620475128575569921</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>1620475128575569921</t>
-        </is>
+      <c r="F89" t="n">
+        <v>1.62047512857557e+18</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -9438,15 +9150,6 @@
           <t>The text suggests a belief in male dominance or advantage, implying men will always prevail or benefit in situations.</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr"/>
       <c r="R89" t="n">
         <v>3091</v>
       </c>
@@ -9497,10 +9200,8 @@
           <t>https://x.com/itsSh0la/status/1620466505115893760</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>1620466505115893760</t>
-        </is>
+      <c r="F90" t="n">
+        <v>1.620466505115894e+18</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -9512,15 +9213,6 @@
           <t>Critique of perceived hypocrisy in feminist demands for equality, highlighting financial expectations in relationships within a Nigerian context.</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
       <c r="R90" t="n">
         <v>3091</v>
       </c>
@@ -9571,10 +9263,8 @@
           <t>https://x.com/itsSh0la/status/1620386661296381955</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>1620386661296381955</t>
-        </is>
+      <c r="F91" t="n">
+        <v>1.620386661296382e+18</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -9586,15 +9276,6 @@
           <t>A tweet expressing a negative opinion about Nigerian men's dating skills.</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
-      <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="n">
         <v>0</v>
       </c>
@@ -9645,10 +9326,8 @@
           <t>https://x.com/itsSh0la/status/1620377121280659459</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>1620377121280659459</t>
-        </is>
+      <c r="F92" t="n">
+        <v>1.620377121280659e+18</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -9660,15 +9339,6 @@
           <t>The text reflects on past relationships, emphasizing emotional control to avoid appearing foolish, despite occasional feelings of longing.</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
       <c r="R92" t="n">
         <v>0</v>
       </c>
@@ -9719,10 +9389,8 @@
           <t>https://x.com/itsSh0la/status/1620034619918921734</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>1620034619918921734</t>
-        </is>
+      <c r="F93" t="n">
+        <v>1.620034619918922e+18</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -9734,15 +9402,6 @@
           <t>A critique of male behavior in relationships, highlighting desperation through actions like excessive texting, financial persuasion, and self-sacrifice for female approval.</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
-      <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
       <c r="R93" t="n">
         <v>0</v>
       </c>
@@ -9793,10 +9452,8 @@
           <t>https://x.com/itsSh0la/status/1619354933362569220</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>1619354933362569220</t>
-        </is>
+      <c r="F94" t="n">
+        <v>1.619354933362569e+18</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -9808,15 +9465,6 @@
           <t>The text emphasizes perseverance and emotional resilience as key traits for achieving goals, highlighting a cultural view of masculinity in Nigeria.</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
-      <c r="P94" t="inlineStr"/>
-      <c r="Q94" t="inlineStr"/>
       <c r="R94" t="n">
         <v>0</v>
       </c>
@@ -9867,10 +9515,8 @@
           <t>https://x.com/itsSh0la/status/1619000891243372544</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>1619000891243372544</t>
-        </is>
+      <c r="F95" t="n">
+        <v>1.619000891243373e+18</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -9882,15 +9528,6 @@
           <t>In Nigerian dating culture, women may request transport fare from men, but genuinely interested women will find their own way to meet.</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
-      <c r="Q95" t="inlineStr"/>
       <c r="R95" t="n">
         <v>0</v>
       </c>
@@ -9941,10 +9578,8 @@
           <t>https://x.com/itsSh0la/status/1618655300382511105</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>1618655300382511105</t>
-        </is>
+      <c r="F96" t="n">
+        <v>1.618655300382511e+18</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -9956,15 +9591,6 @@
           <t>In Nigeria, women often attribute financial struggles to not having a boyfriend, highlighting societal expectations and gender dynamics.</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
       <c r="R96" t="n">
         <v>0</v>
       </c>
@@ -10015,10 +9641,8 @@
           <t>https://x.com/itsSh0la/status/1618258019317604355</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>1618258019317604355</t>
-        </is>
+      <c r="F97" t="n">
+        <v>1.618258019317604e+18</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -10030,15 +9654,6 @@
           <t>Advice for men to reject financial responsibility for entitled women, suggesting women should fend for themselves through begging or other means.</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr"/>
       <c r="R97" t="n">
         <v>3854</v>
       </c>
@@ -10089,10 +9704,8 @@
           <t>https://x.com/itsSh0la/status/1618256715186831361</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>1618256715186831361</t>
-        </is>
+      <c r="F98" t="n">
+        <v>1.618256715186831e+18</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -10104,15 +9717,6 @@
           <t>A girl criticizes a guy's car despite her lower status, highlighting audacity and social dynamics in Nigerian gender interactions.</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
-      <c r="P98" t="inlineStr"/>
-      <c r="Q98" t="inlineStr"/>
       <c r="R98" t="n">
         <v>3854</v>
       </c>
@@ -10163,10 +9767,8 @@
           <t>https://x.com/itsSh0la/status/1618239180903174149</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>1618239180903174149</t>
-        </is>
+      <c r="F99" t="n">
+        <v>1.618239180903174e+18</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -10178,15 +9780,6 @@
           <t>The text suggests that a girl with a certain mindset is considered problematic or 'damaged,' indicating a negative judgment or stereotype.</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
-      <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="n">
         <v>0</v>
       </c>
@@ -10237,10 +9830,8 @@
           <t>https://x.com/jon_d_doe/status/1686113646470901760</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>1686113646470901760</t>
-        </is>
+      <c r="F100" t="n">
+        <v>1.686113646470902e+18</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -10343,10 +9934,8 @@
           <t>https://x.com/jon_d_doe/status/1686081505393553408</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>1686081505393553408</t>
-        </is>
+      <c r="F101" t="n">
+        <v>1.686081505393553e+18</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -10449,10 +10038,8 @@
           <t>https://x.com/jon_d_doe/status/1674877960300511234</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>1674877960300511234</t>
-        </is>
+      <c r="F102" t="n">
+        <v>1.674877960300511e+18</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -10555,10 +10142,8 @@
           <t>https://x.com/jon_d_doe/status/1674876125061816321</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>1674876125061816321</t>
-        </is>
+      <c r="F103" t="n">
+        <v>1.674876125061816e+18</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -10661,10 +10246,8 @@
           <t>https://x.com/jon_d_doe/status/1674869498929635350</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>1674869498929635350</t>
-        </is>
+      <c r="F104" t="n">
+        <v>1.674869498929635e+18</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -10767,10 +10350,8 @@
           <t>https://x.com/jon_d_doe/status/1674856675990200329</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>1674856675990200329</t>
-        </is>
+      <c r="F105" t="n">
+        <v>1.6748566759902e+18</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -10873,10 +10454,8 @@
           <t>https://x.com/jon_d_doe/status/1674854532285620224</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>1674854532285620224</t>
-        </is>
+      <c r="F106" t="n">
+        <v>1.67485453228562e+18</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -10979,10 +10558,8 @@
           <t>https://x.com/jon_d_doe/status/1664013082002092033</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>1664013082002092033</t>
-        </is>
+      <c r="F107" t="n">
+        <v>1.664013082002092e+18</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -11085,10 +10662,8 @@
           <t>https://x.com/jon_d_doe/status/1663979405817856006</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>1663979405817856006</t>
-        </is>
+      <c r="F108" t="n">
+        <v>1.663979405817856e+18</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -11191,10 +10766,8 @@
           <t>https://x.com/jon_d_doe/status/1663974406429843456</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>1663974406429843456</t>
-        </is>
+      <c r="F109" t="n">
+        <v>1.663974406429843e+18</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -11297,10 +10870,8 @@
           <t>https://x.com/jon_d_doe/status/1663973546870095875</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>1663973546870095875</t>
-        </is>
+      <c r="F110" t="n">
+        <v>1.663973546870096e+18</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -11403,10 +10974,8 @@
           <t>https://x.com/jon_d_doe/status/1663872465410334720</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>1663872465410334720</t>
-        </is>
+      <c r="F111" t="n">
+        <v>1.663872465410335e+18</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -11509,10 +11078,8 @@
           <t>https://x.com/jon_d_doe/status/1663830983601266688</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>1663830983601266688</t>
-        </is>
+      <c r="F112" t="n">
+        <v>1.663830983601267e+18</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -11615,10 +11182,8 @@
           <t>https://x.com/jon_d_doe/status/1663822494107590656</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>1663822494107590656</t>
-        </is>
+      <c r="F113" t="n">
+        <v>1.663822494107591e+18</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -11721,10 +11286,8 @@
           <t>https://x.com/jon_d_doe/status/1663818948503060480</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>1663818948503060480</t>
-        </is>
+      <c r="F114" t="n">
+        <v>1.66381894850306e+18</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -11827,10 +11390,8 @@
           <t>https://x.com/jon_d_doe/status/1663801008604995584</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>1663801008604995584</t>
-        </is>
+      <c r="F115" t="n">
+        <v>1.663801008604996e+18</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -11933,10 +11494,8 @@
           <t>https://x.com/jon_d_doe/status/1663628568440582147</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>1663628568440582147</t>
-        </is>
+      <c r="F116" t="n">
+        <v>1.663628568440582e+18</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -12039,10 +11598,8 @@
           <t>https://x.com/jon_d_doe/status/1663626533565497346</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>1663626533565497346</t>
-        </is>
+      <c r="F117" t="n">
+        <v>1.663626533565497e+18</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -12145,10 +11702,8 @@
           <t>https://x.com/jon_d_doe/status/1652779124778315777</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>1652779124778315777</t>
-        </is>
+      <c r="F118" t="n">
+        <v>1.652779124778316e+18</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -12251,10 +11806,8 @@
           <t>https://x.com/jon_d_doe/status/1652761869009010688</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>1652761869009010688</t>
-        </is>
+      <c r="F119" t="n">
+        <v>1.652761869009011e+18</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -12357,10 +11910,8 @@
           <t>https://x.com/jon_d_doe/status/1652759441123553280</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>1652759441123553280</t>
-        </is>
+      <c r="F120" t="n">
+        <v>1.652759441123553e+18</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -12463,10 +12014,8 @@
           <t>https://x.com/jon_d_doe/status/1652752531469004802</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>1652752531469004802</t>
-        </is>
+      <c r="F121" t="n">
+        <v>1.652752531469005e+18</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -12569,10 +12118,8 @@
           <t>https://x.com/jon_d_doe/status/1652668333668327426</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>1652668333668327426</t>
-        </is>
+      <c r="F122" t="n">
+        <v>1.652668333668327e+18</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -12675,10 +12222,8 @@
           <t>https://x.com/jon_d_doe/status/1652592217830174722</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>1652592217830174722</t>
-        </is>
+      <c r="F123" t="n">
+        <v>1.652592217830175e+18</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -12781,10 +12326,8 @@
           <t>https://x.com/jon_d_doe/status/1641321315909922816</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>1641321315909922816</t>
-        </is>
+      <c r="F124" t="n">
+        <v>1.641321315909923e+18</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -12887,10 +12430,8 @@
           <t>https://x.com/jon_d_doe/status/1641315964141682688</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>1641315964141682688</t>
-        </is>
+      <c r="F125" t="n">
+        <v>1.641315964141683e+18</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -12993,10 +12534,8 @@
           <t>https://x.com/jon_d_doe/status/1641174459674402816</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>1641174459674402816</t>
-        </is>
+      <c r="F126" t="n">
+        <v>1.641174459674403e+18</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -13099,10 +12638,8 @@
           <t>https://x.com/jon_d_doe/status/1641155860255653914</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>1641155860255653914</t>
-        </is>
+      <c r="F127" t="n">
+        <v>1.641155860255654e+18</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -13205,10 +12742,8 @@
           <t>https://x.com/jon_d_doe/status/1641047468832968706</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>1641047468832968706</t>
-        </is>
+      <c r="F128" t="n">
+        <v>1.641047468832969e+18</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -13311,10 +12846,8 @@
           <t>https://x.com/jon_d_doe/status/1620540014445858817</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>1620540014445858817</t>
-        </is>
+      <c r="F129" t="n">
+        <v>1.620540014445859e+18</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -13417,10 +12950,8 @@
           <t>https://x.com/jon_d_doe/status/1620530919324123136</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>1620530919324123136</t>
-        </is>
+      <c r="F130" t="n">
+        <v>1.620530919324123e+18</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -13523,10 +13054,8 @@
           <t>https://x.com/jon_d_doe/status/1620526658288754688</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>1620526658288754688</t>
-        </is>
+      <c r="F131" t="n">
+        <v>1.620526658288755e+18</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -13629,10 +13158,8 @@
           <t>https://x.com/jon_d_doe/status/1620496527683899392</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>1620496527683899392</t>
-        </is>
+      <c r="F132" t="n">
+        <v>1.620496527683899e+18</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -13735,10 +13262,8 @@
           <t>https://x.com/jon_d_doe/status/1620469226896248832</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>1620469226896248832</t>
-        </is>
+      <c r="F133" t="n">
+        <v>1.620469226896249e+18</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -13841,10 +13366,8 @@
           <t>https://x.com/jon_d_doe/status/1620401683191992324</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>1620401683191992324</t>
-        </is>
+      <c r="F134" t="n">
+        <v>1.620401683191992e+18</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -13947,10 +13470,8 @@
           <t>https://x.com/jon_d_doe/status/1620368805393465344</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>1620368805393465344</t>
-        </is>
+      <c r="F135" t="n">
+        <v>1.620368805393465e+18</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -14053,10 +13574,8 @@
           <t>https://x.com/jon_d_doe/status/1620328531157991429</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>1620328531157991429</t>
-        </is>
+      <c r="F136" t="n">
+        <v>1.620328531157991e+18</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -14159,10 +13678,8 @@
           <t>https://x.com/jon_d_doe/status/1641155845353291780</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>1641155845353291780</t>
-        </is>
+      <c r="F137" t="n">
+        <v>1.641155845353292e+18</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -14174,15 +13691,6 @@
           <t>The text discusses a perceived change in a woman's behavior in marriage, questioning her loss of respectfulness and submissiveness.</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
-      <c r="L137" t="inlineStr"/>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
-      <c r="P137" t="inlineStr"/>
-      <c r="Q137" t="inlineStr"/>
       <c r="R137" t="n">
         <v>4580</v>
       </c>
@@ -14233,10 +13741,8 @@
           <t>https://x.com/jon_d_doe/status/1641155820632043521</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>1641155820632043521</t>
-        </is>
+      <c r="F138" t="n">
+        <v>1.641155820632044e+18</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -14248,15 +13754,6 @@
           <t>The speaker reflects on life choices, emphasizing confidence in choosing his wife while acknowledging gender dynamics in their relationship.</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
-      <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="inlineStr"/>
       <c r="R138" t="n">
         <v>4580</v>
       </c>
@@ -14307,10 +13804,8 @@
           <t>https://x.com/jon_d_doe/status/1641097671443087360</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>1641097671443087360</t>
-        </is>
+      <c r="F139" t="n">
+        <v>1.641097671443087e+18</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -14322,15 +13817,6 @@
           <t>A metaphorical warning about relationship dynamics, suggesting that repeated mistakes can lead to significant conflict with one's partner.</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
-      <c r="P139" t="inlineStr"/>
-      <c r="Q139" t="inlineStr"/>
       <c r="R139" t="n">
         <v>0</v>
       </c>
@@ -14381,10 +13867,8 @@
           <t>https://x.com/jon_d_doe/status/1641087676420960258</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>1641087676420960258</t>
-        </is>
+      <c r="F140" t="n">
+        <v>1.64108767642096e+18</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -14396,15 +13880,6 @@
           <t>A discussion on property ownership in marriage, highlighting differing opinions between experienced and inexperienced individuals, with a focus on Nigerian cultural norms.</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
-      <c r="P140" t="inlineStr"/>
-      <c r="Q140" t="inlineStr"/>
       <c r="R140" t="n">
         <v>0</v>
       </c>
@@ -14455,10 +13930,8 @@
           <t>https://x.com/jon_d_doe/status/1620368773386756096</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>1620368773386756096</t>
-        </is>
+      <c r="F141" t="n">
+        <v>1.620368773386756e+18</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -14470,15 +13943,6 @@
           <t>The text discusses societal perceptions of women involved in casual relationships in Nigeria, questioning their potential as wives and mothers.</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
-      <c r="M141" t="inlineStr"/>
-      <c r="N141" t="inlineStr"/>
-      <c r="O141" t="inlineStr"/>
-      <c r="P141" t="inlineStr"/>
-      <c r="Q141" t="inlineStr"/>
       <c r="R141" t="n">
         <v>0</v>
       </c>
@@ -14529,10 +13993,8 @@
           <t>https://x.com/jon_d_doe/status/1620368770975006721</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>1620368770975006721</t>
-        </is>
+      <c r="F142" t="n">
+        <v>1.620368770975007e+18</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -14544,15 +14006,6 @@
           <t>A cautionary statement advising men against marrying women with a promiscuous past, suggesting potential future blame and relationship issues.</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
-      <c r="M142" t="inlineStr"/>
-      <c r="N142" t="inlineStr"/>
-      <c r="O142" t="inlineStr"/>
-      <c r="P142" t="inlineStr"/>
-      <c r="Q142" t="inlineStr"/>
       <c r="R142" t="n">
         <v>0</v>
       </c>
@@ -14603,10 +14056,8 @@
           <t>https://x.com/jon_d_doe/status/1620340976228388867</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>1620340976228388867</t>
-        </is>
+      <c r="F143" t="n">
+        <v>1.620340976228389e+18</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -14618,15 +14069,6 @@
           <t>A social media post prompts debate on whether a former prostitute can be a good wife and mother, seeking opinions and reasons.</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
-      <c r="P143" t="inlineStr"/>
-      <c r="Q143" t="inlineStr"/>
       <c r="R143" t="n">
         <v>0</v>
       </c>
@@ -14677,10 +14119,8 @@
           <t>https://x.com/jon_d_doe/status/1663996285093834754</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>1663996285093834754</t>
-        </is>
+      <c r="F144" t="n">
+        <v>1.663996285093835e+18</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -14692,15 +14132,6 @@
           <t>Merged Agba thread (8 consecutive tweets) — women cracking / vetting / man becoming-too-comfortable</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
-      <c r="O144" t="inlineStr"/>
-      <c r="P144" t="inlineStr"/>
-      <c r="Q144" t="inlineStr"/>
       <c r="R144" t="n">
         <v>0</v>
       </c>
@@ -14751,10 +14182,8 @@
           <t>https://x.com/jon_d_doe/status/1663996251531014145</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>1663996251531014145</t>
-        </is>
+      <c r="F145" t="n">
+        <v>1.663996251531014e+18</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -14766,15 +14195,6 @@
           <t>Agba John Doe discusses the role of money in marriage, emphasizing its importance for sustaining relationships and earning respect.</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
-      <c r="L145" t="inlineStr"/>
-      <c r="M145" t="inlineStr"/>
-      <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr"/>
-      <c r="P145" t="inlineStr"/>
-      <c r="Q145" t="inlineStr"/>
       <c r="R145" t="n">
         <v>0</v>
       </c>
@@ -14825,10 +14245,8 @@
           <t>https://x.com/jon_d_doe/status/1663996245789089794</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>1663996245789089794</t>
-        </is>
+      <c r="F146" t="n">
+        <v>1.66399624578909e+18</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -14840,15 +14258,6 @@
           <t>Agba John Doe reflects on his marriage, choosing not to highlight negatives, and credits grace for his leadership.</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
-      <c r="M146" t="inlineStr"/>
-      <c r="N146" t="inlineStr"/>
-      <c r="O146" t="inlineStr"/>
-      <c r="P146" t="inlineStr"/>
-      <c r="Q146" t="inlineStr"/>
       <c r="R146" t="n">
         <v>0</v>
       </c>
@@ -14899,10 +14308,8 @@
           <t>https://x.com/jon_d_doe/status/1663980911627517962</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>1663980911627517962</t>
-        </is>
+      <c r="F147" t="n">
+        <v>1.663980911627518e+18</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -14914,15 +14321,6 @@
           <t>A man praises his wife for supporting them financially during their three-year marriage while he is unemployed.</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
-      <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
-      <c r="O147" t="inlineStr"/>
-      <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="inlineStr"/>
       <c r="R147" t="n">
         <v>0</v>
       </c>
@@ -14973,10 +14371,8 @@
           <t>https://x.com/jon_d_doe/status/1663979994899464203</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>1663979994899464203</t>
-        </is>
+      <c r="F148" t="n">
+        <v>1.663979994899464e+18</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -14988,15 +14384,6 @@
           <t>Agba John Doe discusses marital strain following job and business loss, prompting readers to explore further via a link.</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
-      <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr"/>
       <c r="R148" t="n">
         <v>0</v>
       </c>
@@ -15047,10 +14434,8 @@
           <t>https://x.com/jon_d_doe/status/1663976426515644417</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>1663976426515644417</t>
-        </is>
+      <c r="F149" t="n">
+        <v>1.663976426515644e+18</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -15062,15 +14447,6 @@
           <t>A man is motivated to improve his financial status as his wife earns significantly more than he does.</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
-      <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr"/>
-      <c r="P149" t="inlineStr"/>
-      <c r="Q149" t="inlineStr"/>
       <c r="R149" t="n">
         <v>0</v>
       </c>
@@ -15121,10 +14497,8 @@
           <t>https://x.com/jon_d_doe/status/1663974891501105152</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>1663974891501105152</t>
-        </is>
+      <c r="F150" t="n">
+        <v>1.663974891501105e+18</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -15136,15 +14510,6 @@
           <t>A man's marriage is failing after his business collapse and his wife leaving, despite marrying into wealth.</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
-      <c r="P150" t="inlineStr"/>
-      <c r="Q150" t="inlineStr"/>
       <c r="R150" t="n">
         <v>0</v>
       </c>
@@ -15195,10 +14560,8 @@
           <t>https://x.com/jon_d_doe/status/1641155849115582478</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>1641155849115582478</t>
-        </is>
+      <c r="F151" t="n">
+        <v>1.641155849115582e+18</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -15210,15 +14573,6 @@
           <t>Merged Agba thread (12 consecutive tweets) — women manipulation / property / leadership</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
-      <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr"/>
-      <c r="P151" t="inlineStr"/>
-      <c r="Q151" t="inlineStr"/>
       <c r="R151" t="n">
         <v>4580</v>
       </c>
@@ -15269,10 +14623,8 @@
           <t>https://x.com/Wizarab10/status/1664054075162341376</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>1664054075162341376</t>
-        </is>
+      <c r="F152" t="n">
+        <v>1.664054075162341e+18</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -15375,10 +14727,8 @@
           <t>https://x.com/Wizarab10/status/1664050449861734417</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>1664050449861734417</t>
-        </is>
+      <c r="F153" t="n">
+        <v>1.664050449861734e+18</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -15481,10 +14831,8 @@
           <t>https://x.com/Wizarab10/status/1664045875650330626</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>1664045875650330626</t>
-        </is>
+      <c r="F154" t="n">
+        <v>1.664045875650331e+18</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -15587,10 +14935,8 @@
           <t>https://x.com/Wizarab10/status/1664023601756897280</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>1664023601756897280</t>
-        </is>
+      <c r="F155" t="n">
+        <v>1.664023601756897e+18</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -15693,10 +15039,8 @@
           <t>https://x.com/Wizarab10/status/1663879826623610881</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>1663879826623610881</t>
-        </is>
+      <c r="F156" t="n">
+        <v>1.663879826623611e+18</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -15750,13 +15094,13 @@
         </is>
       </c>
       <c r="R156" t="n">
-        <v>0</v>
+        <v>433</v>
       </c>
       <c r="S156" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="T156" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="U156" t="n">
         <v>0</v>
@@ -15799,10 +15143,8 @@
           <t>https://x.com/Wizarab10/status/1663878777707847682</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>1663878777707847682</t>
-        </is>
+      <c r="F157" t="n">
+        <v>1.663878777707848e+18</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -15905,10 +15247,8 @@
           <t>https://x.com/Wizarab10/status/1663864642567917569</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>1663864642567917569</t>
-        </is>
+      <c r="F158" t="n">
+        <v>1.663864642567918e+18</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -16011,10 +15351,8 @@
           <t>https://x.com/Wizarab10/status/1663863231159345154</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>1663863231159345154</t>
-        </is>
+      <c r="F159" t="n">
+        <v>1.663863231159345e+18</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -16117,10 +15455,8 @@
           <t>https://x.com/Wizarab10/status/1663849151526850561</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>1663849151526850561</t>
-        </is>
+      <c r="F160" t="n">
+        <v>1.663849151526851e+18</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -16223,10 +15559,8 @@
           <t>https://x.com/Wizarab10/status/1663681443803930624</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>1663681443803930624</t>
-        </is>
+      <c r="F161" t="n">
+        <v>1.663681443803931e+18</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -16329,10 +15663,8 @@
           <t>https://x.com/Wizarab10/status/1652792458181263360</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>1652792458181263360</t>
-        </is>
+      <c r="F162" t="n">
+        <v>1.652792458181263e+18</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -16435,10 +15767,8 @@
           <t>https://x.com/Wizarab10/status/1652789430443180032</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>1652789430443180032</t>
-        </is>
+      <c r="F163" t="n">
+        <v>1.65278943044318e+18</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -16541,10 +15871,8 @@
           <t>https://x.com/Wizarab10/status/1652786591478194176</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>1652786591478194176</t>
-        </is>
+      <c r="F164" t="n">
+        <v>1.652786591478194e+18</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -16647,10 +15975,8 @@
           <t>https://x.com/Wizarab10/status/1652778262702039048</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>1652778262702039048</t>
-        </is>
+      <c r="F165" t="n">
+        <v>1.652778262702039e+18</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -16753,10 +16079,8 @@
           <t>https://x.com/Wizarab10/status/1652775309014446081</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>1652775309014446081</t>
-        </is>
+      <c r="F166" t="n">
+        <v>1.652775309014446e+18</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -16859,10 +16183,8 @@
           <t>https://x.com/Wizarab10/status/1652759568479588352</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>1652759568479588352</t>
-        </is>
+      <c r="F167" t="n">
+        <v>1.652759568479588e+18</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -16965,10 +16287,8 @@
           <t>https://x.com/Wizarab10/status/1652758073541292032</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>1652758073541292032</t>
-        </is>
+      <c r="F168" t="n">
+        <v>1.652758073541292e+18</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -17071,10 +16391,8 @@
           <t>https://x.com/Wizarab10/status/1652730128177278980</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>1652730128177278980</t>
-        </is>
+      <c r="F169" t="n">
+        <v>1.652730128177279e+18</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -17177,10 +16495,8 @@
           <t>https://x.com/Wizarab10/status/1652653921628823554</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>1652653921628823554</t>
-        </is>
+      <c r="F170" t="n">
+        <v>1.652653921628824e+18</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -17283,10 +16599,8 @@
           <t>https://x.com/Wizarab10/status/1652637832043790337</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>1652637832043790337</t>
-        </is>
+      <c r="F171" t="n">
+        <v>1.65263783204379e+18</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -17389,10 +16703,8 @@
           <t>https://x.com/Wizarab10/status/1652632250100350977</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>1652632250100350977</t>
-        </is>
+      <c r="F172" t="n">
+        <v>1.652632250100351e+18</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -17495,10 +16807,8 @@
           <t>https://x.com/Wizarab10/status/1652613708361736194</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>1652613708361736194</t>
-        </is>
+      <c r="F173" t="n">
+        <v>1.652613708361736e+18</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -17601,10 +16911,8 @@
           <t>https://x.com/Wizarab10/status/1652613172400988160</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>1652613172400988160</t>
-        </is>
+      <c r="F174" t="n">
+        <v>1.652613172400988e+18</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -17707,10 +17015,8 @@
           <t>https://x.com/Wizarab10/status/1652611840378126336</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>1652611840378126336</t>
-        </is>
+      <c r="F175" t="n">
+        <v>1.652611840378126e+18</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -17813,10 +17119,8 @@
           <t>https://x.com/Wizarab10/status/1652610742292561921</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>1652610742292561921</t>
-        </is>
+      <c r="F176" t="n">
+        <v>1.652610742292562e+18</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -17919,10 +17223,8 @@
           <t>https://x.com/Wizarab10/status/1652610743580217344</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>1652610743580217344</t>
-        </is>
+      <c r="F177" t="n">
+        <v>1.652610743580217e+18</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -18025,10 +17327,8 @@
           <t>https://x.com/Wizarab10/status/1652607935829123072</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>1652607935829123072</t>
-        </is>
+      <c r="F178" t="n">
+        <v>1.652607935829123e+18</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -18131,10 +17431,8 @@
           <t>https://x.com/Wizarab10/status/1652606997215182850</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>1652606997215182850</t>
-        </is>
+      <c r="F179" t="n">
+        <v>1.652606997215183e+18</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -18237,10 +17535,8 @@
           <t>https://x.com/Wizarab10/status/1652605299235119104</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>1652605299235119104</t>
-        </is>
+      <c r="F180" t="n">
+        <v>1.652605299235119e+18</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -18343,10 +17639,8 @@
           <t>https://x.com/Wizarab10/status/1652604814889570304</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>1652604814889570304</t>
-        </is>
+      <c r="F181" t="n">
+        <v>1.65260481488957e+18</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -18449,10 +17743,8 @@
           <t>https://x.com/Wizarab10/status/1652603868771938306</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr">
-        <is>
-          <t>1652603868771938306</t>
-        </is>
+      <c r="F182" t="n">
+        <v>1.652603868771938e+18</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -18555,10 +17847,8 @@
           <t>https://x.com/Wizarab10/status/1652600422668828672</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>1652600422668828672</t>
-        </is>
+      <c r="F183" t="n">
+        <v>1.652600422668829e+18</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -18661,10 +17951,8 @@
           <t>https://x.com/Wizarab10/status/1652597521510744064</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>1652597521510744064</t>
-        </is>
+      <c r="F184" t="n">
+        <v>1.652597521510744e+18</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -18767,10 +18055,8 @@
           <t>https://x.com/Wizarab10/status/1641887533855395854</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr">
-        <is>
-          <t>1641887533855395854</t>
-        </is>
+      <c r="F185" t="n">
+        <v>1.641887533855396e+18</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -18873,10 +18159,8 @@
           <t>https://x.com/Wizarab10/status/1641855732931756033</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>1641855732931756033</t>
-        </is>
+      <c r="F186" t="n">
+        <v>1.641855732931756e+18</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -18979,10 +18263,8 @@
           <t>https://x.com/Wizarab10/status/1641800899814121474</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
-        <is>
-          <t>1641800899814121474</t>
-        </is>
+      <c r="F187" t="n">
+        <v>1.641800899814121e+18</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -19085,10 +18367,8 @@
           <t>https://x.com/Wizarab10/status/1641792600863645696</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr">
-        <is>
-          <t>1641792600863645696</t>
-        </is>
+      <c r="F188" t="n">
+        <v>1.641792600863646e+18</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -19191,10 +18471,8 @@
           <t>https://x.com/Wizarab10/status/1641787210054660097</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr">
-        <is>
-          <t>1641787210054660097</t>
-        </is>
+      <c r="F189" t="n">
+        <v>1.64178721005466e+18</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -19297,10 +18575,8 @@
           <t>https://x.com/Wizarab10/status/1641780775753269248</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr">
-        <is>
-          <t>1641780775753269248</t>
-        </is>
+      <c r="F190" t="n">
+        <v>1.641780775753269e+18</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -19354,13 +18630,13 @@
         </is>
       </c>
       <c r="R190" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="S190" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="T190" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U190" t="n">
         <v>0</v>
@@ -19403,10 +18679,8 @@
           <t>https://x.com/Wizarab10/status/1641780741360025602</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>1641780741360025602</t>
-        </is>
+      <c r="F191" t="n">
+        <v>1.641780741360026e+18</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -19509,10 +18783,8 @@
           <t>https://x.com/Wizarab10/status/1641776275877507073</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>1641776275877507073</t>
-        </is>
+      <c r="F192" t="n">
+        <v>1.641776275877507e+18</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -19524,15 +18796,6 @@
           <t>Wizarab defends manipulation as distinct from coercion, emphasizing personal responsibility and criticizing those who conflate the two.</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
-      <c r="M192" t="inlineStr"/>
-      <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
-      <c r="P192" t="inlineStr"/>
-      <c r="Q192" t="inlineStr"/>
       <c r="R192" t="n">
         <v>457</v>
       </c>
@@ -19583,10 +18846,8 @@
           <t>https://x.com/Wizarab10/status/1641760900993495041</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr">
-        <is>
-          <t>1641760900993495041</t>
-        </is>
+      <c r="F193" t="n">
+        <v>1.641760900993495e+18</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -19598,15 +18859,6 @@
           <t>Wizarab points out that women also seek sex, challenging gendered assumptions about sexual pursuit.</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
-      <c r="O193" t="inlineStr"/>
-      <c r="P193" t="inlineStr"/>
-      <c r="Q193" t="inlineStr"/>
       <c r="R193" t="n">
         <v>0</v>
       </c>
@@ -19657,10 +18909,8 @@
           <t>https://x.com/Wizarab10/status/1619650876221829121</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>1619650876221829121</t>
-        </is>
+      <c r="F194" t="n">
+        <v>1.619650876221829e+18</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -19672,15 +18922,6 @@
           <t>The tweet describes leaving a woman after a brief encounter to avoid commitment when she seeks relationship clarity.</t>
         </is>
       </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
-      <c r="M194" t="inlineStr"/>
-      <c r="N194" t="inlineStr"/>
-      <c r="O194" t="inlineStr"/>
-      <c r="P194" t="inlineStr"/>
-      <c r="Q194" t="inlineStr"/>
       <c r="R194" t="n">
         <v>480</v>
       </c>
@@ -19731,10 +18972,8 @@
           <t>https://x.com/Wizarab10/status/1620358713474433024</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
-        <is>
-          <t>1620358713474433024</t>
-        </is>
+      <c r="F195" t="n">
+        <v>1.620358713474433e+18</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -19746,15 +18985,6 @@
           <t>The tweet suggests skepticism about equality, using a metaphor about urinating in one place to highlight collective action or unity.</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
-      <c r="M195" t="inlineStr"/>
-      <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
-      <c r="P195" t="inlineStr"/>
-      <c r="Q195" t="inlineStr"/>
       <c r="R195" t="n">
         <v>61</v>
       </c>
@@ -19805,10 +19035,8 @@
           <t>https://x.com/Wizarab10/status/1664037638863454208</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr">
-        <is>
-          <t>1664037638863454208</t>
-        </is>
+      <c r="F196" t="n">
+        <v>1.664037638863454e+18</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -19820,15 +19048,6 @@
           <t>Focus on finding the right fit for your life, not on the quantity of options available.</t>
         </is>
       </c>
-      <c r="I196" t="inlineStr"/>
-      <c r="J196" t="inlineStr"/>
-      <c r="K196" t="inlineStr"/>
-      <c r="L196" t="inlineStr"/>
-      <c r="M196" t="inlineStr"/>
-      <c r="N196" t="inlineStr"/>
-      <c r="O196" t="inlineStr"/>
-      <c r="P196" t="inlineStr"/>
-      <c r="Q196" t="inlineStr"/>
       <c r="R196" t="n">
         <v>85</v>
       </c>
@@ -19879,10 +19098,8 @@
           <t>https://x.com/Wizarab10/status/1663858197310865409</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr">
-        <is>
-          <t>1663858197310865409</t>
-        </is>
+      <c r="F197" t="n">
+        <v>1.663858197310865e+18</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -19894,15 +19111,6 @@
           <t>The text discusses evaluating compatibility in relationships and deciding to leave if the relationship is not suitable.</t>
         </is>
       </c>
-      <c r="I197" t="inlineStr"/>
-      <c r="J197" t="inlineStr"/>
-      <c r="K197" t="inlineStr"/>
-      <c r="L197" t="inlineStr"/>
-      <c r="M197" t="inlineStr"/>
-      <c r="N197" t="inlineStr"/>
-      <c r="O197" t="inlineStr"/>
-      <c r="P197" t="inlineStr"/>
-      <c r="Q197" t="inlineStr"/>
       <c r="R197" t="n">
         <v>45</v>
       </c>
@@ -19953,10 +19161,8 @@
           <t>https://x.com/Wizarab10/status/1663852815511429120</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>1663852815511429120</t>
-        </is>
+      <c r="F198" t="n">
+        <v>1.663852815511429e+18</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -19968,15 +19174,6 @@
           <t>The text discusses ending relationships, skepticism about swearing on the Bible, and accepting the love one believes they deserve.</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr"/>
-      <c r="J198" t="inlineStr"/>
-      <c r="K198" t="inlineStr"/>
-      <c r="L198" t="inlineStr"/>
-      <c r="M198" t="inlineStr"/>
-      <c r="N198" t="inlineStr"/>
-      <c r="O198" t="inlineStr"/>
-      <c r="P198" t="inlineStr"/>
-      <c r="Q198" t="inlineStr"/>
       <c r="R198" t="n">
         <v>86</v>
       </c>
@@ -20027,10 +19224,8 @@
           <t>https://x.com/Wizarab10/status/1663817389069283328</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
-        <is>
-          <t>1663817389069283328</t>
-        </is>
+      <c r="F199" t="n">
+        <v>1.663817389069283e+18</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -20042,15 +19237,6 @@
           <t>The text discusses the thrill of chasing in relationships, emphasizing it's unrelated to personal value and varies among individuals.</t>
         </is>
       </c>
-      <c r="I199" t="inlineStr"/>
-      <c r="J199" t="inlineStr"/>
-      <c r="K199" t="inlineStr"/>
-      <c r="L199" t="inlineStr"/>
-      <c r="M199" t="inlineStr"/>
-      <c r="N199" t="inlineStr"/>
-      <c r="O199" t="inlineStr"/>
-      <c r="P199" t="inlineStr"/>
-      <c r="Q199" t="inlineStr"/>
       <c r="R199" t="n">
         <v>111</v>
       </c>
@@ -20101,10 +19287,8 @@
           <t>https://x.com/Wizarab10/status/1652613288054726657</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr">
-        <is>
-          <t>1652613288054726657</t>
-        </is>
+      <c r="F200" t="n">
+        <v>1.652613288054727e+18</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -20116,15 +19300,6 @@
           <t>The text highlights the significance of sex as a crucial factor in a given context.</t>
         </is>
       </c>
-      <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr"/>
-      <c r="K200" t="inlineStr"/>
-      <c r="L200" t="inlineStr"/>
-      <c r="M200" t="inlineStr"/>
-      <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr"/>
-      <c r="P200" t="inlineStr"/>
-      <c r="Q200" t="inlineStr"/>
       <c r="R200" t="n">
         <v>0</v>
       </c>
@@ -20175,10 +19350,8 @@
           <t>https://x.com/Wizarab10/status/1652599667190906881</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
-        <is>
-          <t>1652599667190906881</t>
-        </is>
+      <c r="F201" t="n">
+        <v>1.652599667190907e+18</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -20190,15 +19363,6 @@
           <t>The text discusses insecurity, body positivity, and the unrealistic pursuit of perfection, particularly in relation to obesity.</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
-      <c r="M201" t="inlineStr"/>
-      <c r="N201" t="inlineStr"/>
-      <c r="O201" t="inlineStr"/>
-      <c r="P201" t="inlineStr"/>
-      <c r="Q201" t="inlineStr"/>
       <c r="R201" t="n">
         <v>0</v>
       </c>
@@ -20249,10 +19413,8 @@
           <t>https://x.com/Wizarab10/status/1641796973115187205</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
-        <is>
-          <t>1641796973115187205</t>
-        </is>
+      <c r="F202" t="n">
+        <v>1.641796973115187e+18</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -20264,15 +19426,6 @@
           <t>The text advises on forming friendships naturally and approaching women confidently, even if shy, emphasizing authenticity and direct communication.</t>
         </is>
       </c>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
-      <c r="M202" t="inlineStr"/>
-      <c r="N202" t="inlineStr"/>
-      <c r="O202" t="inlineStr"/>
-      <c r="P202" t="inlineStr"/>
-      <c r="Q202" t="inlineStr"/>
       <c r="R202" t="n">
         <v>57</v>
       </c>
@@ -20323,10 +19476,8 @@
           <t>https://x.com/Wizarab10/status/1641778203978088448</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr">
-        <is>
-          <t>1641778203978088448</t>
-        </is>
+      <c r="F203" t="n">
+        <v>1.641778203978088e+18</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -20338,15 +19489,6 @@
           <t>A cautionary message about the dangers in the world, urging protection of loved ones from harmful individuals.</t>
         </is>
       </c>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
-      <c r="M203" t="inlineStr"/>
-      <c r="N203" t="inlineStr"/>
-      <c r="O203" t="inlineStr"/>
-      <c r="P203" t="inlineStr"/>
-      <c r="Q203" t="inlineStr"/>
       <c r="R203" t="n">
         <v>33</v>
       </c>
@@ -20397,10 +19539,8 @@
           <t>https://x.com/Wizarab10/status/1619731584768442368</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>1619731584768442368</t>
-        </is>
+      <c r="F204" t="n">
+        <v>1.619731584768442e+18</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -20412,15 +19552,6 @@
           <t>A statement expressing criticism towards a man for not managing his responsibilities independently, implying societal expectations of male competence.</t>
         </is>
       </c>
-      <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
-      <c r="M204" t="inlineStr"/>
-      <c r="N204" t="inlineStr"/>
-      <c r="O204" t="inlineStr"/>
-      <c r="P204" t="inlineStr"/>
-      <c r="Q204" t="inlineStr"/>
       <c r="R204" t="n">
         <v>102</v>
       </c>
@@ -20762,9 +19893,6 @@
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -20807,9 +19935,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -20880,9 +20005,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -20918,9 +20040,6 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -20963,9 +20082,6 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -20980,9 +20096,6 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -20990,9 +20103,6 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -21034,9 +20144,6 @@
           <t xml:space="preserve">  - Group by misogyny level → compare engagement distributions</t>
         </is>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">

</xml_diff>